<commit_message>
refactor: rename UE TableDesk to UERowForge with compatible settings
</commit_message>
<xml_diff>
--- a/Tool/resources/TableTemplate.xlsx
+++ b/Tool/resources/TableTemplate.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Guide" sheetId="1" r:id="Rcb845923704844b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="2" r:id="R704581c1ab6c411c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="3" r:id="Rdec32e5980884b74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Guide" sheetId="1" r:id="R6359eda5a71d4f6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="2" r:id="R9d38225fb4344d09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="3" r:id="R733710a4568d4846"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -409,7 +409,7 @@
   <x:sheetData>
     <x:row r="1" ht="40" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>UE TableDesk · Excel template</x:v>
+        <x:v>UERowForge · Excel template</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>

</xml_diff>